<commit_message>
Move the game's own text into a workbook checked against the framework
- engine: every player-facing string now comes from "HEARsay game text.xlsx"
  (Passages, Text, Facts); the engine holds no wording. New game_text.py and
  check_framework.py check the workbook against an export of the framework
  doc: passage names, cited sections, verbatim text and the framework's numbers.
- matrix: scenario text is filed under the framework's passage names
  (the Hook, Start, Submission, ending), plus Mystery and Final-answer form
  sheets; the question budget now comes from the framework facts.
- final-answer questions ("Who removed it?") moved from the engine to the matrix.
- text: "Acknowledge the other's perspective" (as in the framework), and the
  first rule no longer says each witness can be interviewed only once.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenario/The Commons' Comma – Response Matrix.xlsx
+++ b/scenario/The Commons' Comma – Response Matrix.xlsx
@@ -9,18 +9,17 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final answer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grid" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long table" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Witnesses" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clues" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major clues" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Red herrings" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Follow-ups" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endings" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constraints" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passages" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mystery" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final-answer form" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grid" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long table" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Witnesses" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clues" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Clues" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Red Herrings" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Follow-ups" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -504,7 +503,7 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>This workbook is the source the game is built from. Edit it here, keep the Scenario Packet in step, then rebuild; the build stops if the workbook breaks a rule or the packet disagrees with it. Sheets marked 'checked' repeat information held elsewhere in the workbook and must match it.</t>
+          <t>This workbook is the scenario the game is built from, in the terms of the framework (the 'HEARsay mysteries' Google Doc). Edit it here, keep the Scenario Packet in step, then rebuild; the build stops if the workbook breaks a framework rule, disagrees with itself, or disagrees with the packet. The framework's numbers (8 witnesses, 20 Clues, the 40-question budget …) live in the Facts sheet of 'HEARsay game text.xlsx' in the Twine engine folder, which is checked against the framework.</t>
         </is>
       </c>
     </row>
@@ -516,151 +515,139 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Title, IDs, question budget, follow-up bonus, map file, play link and the pitch shown on the game's start screen.</t>
+          <t>Title, scenario ID, Twine IFID, map file and play link.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Passages</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>The mystery, the solution, the player's role, the president's briefing and the controversy text the game shows.</t>
+          <t>The scenario's own text for the framework's passages: the Start summary, the Hook (situation, assignment, the CCC), the out-of-questions message on Submission, and the ending for each verdict. Everything else on screen is the game's own text.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Final answer</t>
+          <t>Mystery</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The people and places offered on the final-answer screen. Mark exactly one of each 'yes' as correct.</t>
+          <t>The mystery (the question the player answers), the solution, and the two questions on the final-answer form.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Grid</t>
+          <t>Final-answer form</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Checked: 8 questions × 8 witnesses, the same answers as the Long table laid out as a grid. TW = tripwire.</t>
+          <t>The people and places offered at the end. Mark exactly one of each 'yes' as correct.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Long table</t>
+          <t>Grid</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>One row per cell (64 rows): the answers the game gives, their item, and whether the opinion is receptive. Tripwire rows hold the walk-away text.</t>
+          <t>Checked copy: the readable condensed version of the Response Matrix (8 questions × 8 witnesses). TW = tripwire.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Witnesses</t>
+          <t>Long table</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Profiles, tripwires, walk-away text and receptiveness ranks. 'Tripwire question' is checked against Questions.</t>
+          <t>The longform Response Matrix the game reads: one row per cell (64 rows), with item, receptive flag and text. Tripwire rows hold the walk-away text.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Questions</t>
+          <t>Witnesses</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The eight shared questions and their tripwire owners.</t>
+          <t>Information, image, ID, position on the CCC, tripwire, walk-away text and receptiveness rank. 'Tripwire question' is checked against Questions.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Clues</t>
+          <t>Questions</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The 20 clues and their Major Clue group. 'Given by' is checked against the Long table.</t>
+          <t>The eight questions and whose tripwire each one is.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Major clues</t>
+          <t>Clues</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>The four Major Clues in reveal order.</t>
+          <t>The 20 Clues and their Major Clue. 'Given by' is checked against the Long table.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Red herrings</t>
+          <t>Major Clues</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>The 16 red herrings and their sets. 'Given by' is checked; set title and resolution must be the same on every row of a set.</t>
+          <t>The four Major Clues in the order they are earned.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Follow-ups</t>
+          <t>Red Herrings</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Per-witness follow-up pairs, explanations and walk-away text.</t>
+          <t>The 16 Red Herrings and their sets. 'Given by' is checked; the set title and how the set is discounted must match on every row of a set.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Endings</t>
+          <t>Follow-ups</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>The text of each ending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Constraints</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>The structural rules the build enforces (for reference).</t>
+          <t>Each witness's follow-up pair, the explanation shown on success, and the walk-away text on failure.</t>
         </is>
       </c>
     </row>
@@ -670,6 +657,488 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Major clue group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Clue</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Given by</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>MC1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>The Charter was in its blue archival folder, seal intact, at the end of the student forum at 7:45 p.m., and was returned to the archive cabinet.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Leo Martinez (Q8); Evan Cho (Q5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>MC1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah's graduate credential opened the archive at 8:42 p.m. It was an ordinary entry; the door and cabinet show no damage.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah (Q1); Priya Nwosu (Q7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>MC1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>The archive access log was edited at 9:17 p.m., after the archive closed at 9:00. Editing the log requires an archive credential, not a maintenance or administrative one.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Priya Nwosu (Q1); Sofia Alvarez (Q5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MC1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>No credential other than Mira's opened the archive between the forum and closing time.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Leo Martinez (Q3); Priya Nwosu (Q6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>MC1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Mira left the archive area at about 8:50 p.m. carrying something flat inside a protective sleeve.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Leo Martinez (Q7); Sofia Alvarez (Q1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>MC2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Mira has argued for months, in seminars and in print, that the disputed mark is an original comma, the reading that gives students a strong veto.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah (Q2); Nia Williams (Q2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>MC2</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>In the newspaper photograph of the 'examination copy', the disputed mark has sharper edges and a different paper shadow than the surrounding ink.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah (Q6); Sofia Alvarez (Q2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>MC2</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>A small crease near the mark, visible in older photographs of the Charter, is absent from the newspaper photograph.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Priya Nwosu (Q3); Sofia Alvarez (Q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MC2</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Late in the preparations the event materials stopped saying 'the original Charter' and started saying 'the Charter'; Celia Park kept pressing for 'a clean answer' for the Board.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Leo Martinez (Q5); Hana Petrov (Q3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>MC2</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Mira told other students she wanted to make sure 'the experts examine the real object', and feared the original would be quietly swapped or lost after the event.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Hana Petrov (Q2); Nia Williams (Q3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>MC3</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>At about 8:50 p.m. Mira asked whether the theatre had a dry, light-proof place to keep paper.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Jonah Reed (Q1); Evan Cho (Q4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>MC3</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Jonah gave Mira an empty poster tube labelled 'Spring Gala 2023'.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Jonah Reed (Q3); Nia Williams (Q4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>MC3</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>At about 8:55 p.m. a long cardboard tube with theatre paint on one end was carried from the Commons toward the theatre.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Leo Martinez (Q4); Evan Cho (Q1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>MC3</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>The 'Spring Gala 2023' tube is now in the theatre scenery loft, and it is heavier than an empty tube should be.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Jonah Reed (Q6); Sofia Alvarez (Q4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>MC3</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>After Mira's visit Jonah moved several tubes in the scenery loft and did not update the inventory sheet.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Jonah Reed (Q8); Hana Petrov (Q4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>MC4</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Mira and Jonah were seen talking near the theatre at about 8:52 p.m. It looked like a practical conversation about storage, not a confrontation.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Evan Cho (Q7); Nia Williams (Q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>MC4</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Mira and Jonah disagree about the renovation's details but share one goal: the Charter must not be damaged or lost.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Jonah Reed (Q2); Hana Petrov (Q7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>MC4</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>The Charter's protective sleeve is missing along with it. Whoever took it handled it like a conservator, not a thief.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah (Q4); Priya Nwosu (Q4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>MC4</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Members of the administrative steering group do not hold archive credentials; they reach the archive through the archivist's office, and none of them used it that night.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah (Q5); Hana Petrov (Q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>MC4</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Mira said she would 'keep it safe until someone can compare the two'. She intends to return the Charter once the examination copy has been checked against it.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Evan Cho (Q3); Nia Williams (Q6)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -825,7 +1294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -860,7 +1329,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Red herring</t>
+          <t>Red Herring</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1391,7 +1860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1701,251 +2170,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="110" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ending</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>When</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>correct</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Right person and right place</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>You name Mira Shah and the theatre scenery loft. The president sends the archivist emeritus, Ruth Halpern, to the loft with you. Inside the 'Spring Gala 2023' tube is the Charter in its protective sleeve. Mira, when found, admits she removed it and edited the log because she believed the examination copy was not the original. Then the hidden payoff: Halpern lays the recovered Charter beside the examination copy. The copy is a near-perfect replica, commissioned at enormous expense by Adrian Vale, Celia Park and Martin Ellison so that the disputed mark would read as a blot and no student vote would ever be required. It was to be displayed in a glass case in the renovated center as though it were the original. The examination goes ahead at six with the real Charter on the table. The replica becomes a historical artifact after all, labelled honestly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>right_person_wrong_place</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Right person, wrong place</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>You identify who removed the Charter but not where it is. The examination begins at six without the original, and the replica is examined as though it were genuine.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>wrong</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Wrong person</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Your explanation does not fit the strongest evidence. The person you named had a motive, but the timeline, the access record and the hiding-place clues point elsewhere. The examination proceeds with the wrong document.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>out_of_questions</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Question budget used up</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>You have used your forty questions. The president needs an answer now.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Constraint</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Witnesses</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Questions</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Tripwires</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>one per witness, one per question (a permutation)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Per witness</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>1 tripwire, 5 clues, 2 red herrings</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Clues</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>20, each given by exactly two witnesses</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Red herrings</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>16, each given once, in cancelling sets of at least two</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Major clues</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>4, five clues each, no overlap</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Receptive answers</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>7,6,5,4,3,2,1,0 by rank = 28 of 56</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Follow-ups</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>one per witness; do not count toward the question budget (Settings)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2020,81 +2251,34 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Question budget</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>40</v>
+          <t>Map</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>campus-map.jpg</t>
+        </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Questions per game. Follow-ups do not count; tripwire questions do.</t>
+          <t>Campus map file in the Assets folder.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Follow-up bonus</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>1</v>
+          <t>Play URL</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>https://holytispoon.github.io/HEARsay-Mysteries-Commons-Comma/</t>
+        </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bonus points for a successful follow-up once all Major Clues are earned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Map</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>campus-map.jpg</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Campus map file in the Assets folder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Play URL</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>https://holytispoon.github.io/HEARsay-Mysteries-Commons-Comma/</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
           <t>The GitHub Pages link, shown at the top of the repository README. Leave blank to omit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Pitch</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>The night before the university publicly examines its founding Charter to settle whether a disputed ink mark is a comma, the Charter vanishes from the archive. You have until five o'clock and forty questions to find out who took it, why, and where it is, by interviewing eight students who each know something and each have an opinion about the renovation the comma would decide.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Shown on the game's start screen.</t>
         </is>
       </c>
     </row>
@@ -2109,120 +2293,266 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Passage</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Text</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mystery</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Who removed the Commons Charter from the university archive last night, why did they do it, and where is it now?</t>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>The night before the university publicly examines its founding Charter to settle whether a disputed ink mark is a comma, the Charter vanishes from the archive. You have until five o'clock and forty questions to find out who took it, why, and where it is, by interviewing eight students who each know something and each have an opinion about the renovation the comma would decide.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Background/summary shown on the title screen.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Solution</t>
+          <t>the Hook</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mira Shah, a graduate archival researcher, removed the Charter using her own legitimate credential at 8:42 p.m., then edited the archive access log at 9:17 p.m. to hide the removal. She did it because she was convinced the document being prepared for tonight's public examination is not the original: the newspaper photograph of the 'examination copy' shows a disputed mark with edges and shadow that do not match the surrounding ink, and a crease visible in older photographs is missing. She hid the Charter, rolled in its protective sleeve, inside a poster tube labelled 'Spring Gala 2023' that Jonah Reed gave her, and the tube is now in the student theatre's scenery loft.</t>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>You have just started a work-study job as an administrative assistant in the Office of the President. You expected calendars, filing and photocopying. At 9:05 a.m. on your first morning the president closes the office door.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Situates the player.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Player role</t>
+          <t>the Hook</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>You have just started a work-study job as an administrative assistant in the Office of the President. You expected calendars, filing and photocopying. At 9:05 a.m. on your first morning the president closes the office door.</t>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>“At six o'clock tonight, the university will publicly examine the Commons Charter. I have just learned that the document prepared for examination may not be the original. If that becomes public before we understand it, the university faces a scandal, and the Board may approve a renovation on the strength of falsified evidence. Find out who removed the Charter, why, and where it is now. Talk to the students who were around the Commons last night. Do not alert the press. You have until five.”</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The task and the time pressure, from whoever gives the mystery. Also in the Case file.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Briefing</t>
+          <t>the Hook</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>“At six o'clock tonight, the university will publicly examine the Commons Charter. I have just learned that the document prepared for examination may not be the original. If that becomes public before we understand it, the university faces a scandal, and the Board may approve a renovation on the strength of falsified evidence. Find out who removed the Charter, why, and where it is now. Talk to the students who were around the Commons last night. Do not alert the press. You have until five.”</t>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>The Commons renovation</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>The Current Campus Controversy's name.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Controversy name</t>
+          <t>the Hook</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The Commons renovation</t>
-        </is>
-      </c>
+          <t>CCC summary</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The university plans to redevelop the historic Student Commons into an 'Innovation and Safety Hub': AI-assisted classrooms, facial-recognition entry, commercial research offices and fewer student-organized spaces. Supporters call it overdue modernization with real safety, accessibility and wellness gains. Opponents call it privatization and surveillance that hands student space to administrators and sponsors. The fight has crystallized around the Commons Charter's veto clause and one disputed mark that may or may not be a comma.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Controversy summary</t>
+          <t>the Hook</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>The university plans to redevelop the historic Student Commons into an 'Innovation and Safety Hub': AI-assisted classrooms, facial-recognition entry, commercial research offices and fewer student-organized spaces. Supporters call it overdue modernization with real safety, accessibility and wellness gains. Opponents call it privatization and surveillance that hands student space to administrators and sponsors. The fight has crystallized around the Commons Charter's veto clause and one disputed mark that may or may not be a comma.</t>
+          <t>Clause</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>“No renovation, alteration, or demolition of the Commons shall proceed without the approval of the University Board of Directors, the President, the Provost, the Faculty Senate, the faculty house masters and students of the University.”</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Optional: a quoted document at the heart of the CCC.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Clause</t>
+          <t>the Hook</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>“No renovation, alteration, or demolition of the Commons shall proceed without the approval of the University Board of Directors, the President, the Provost, the Faculty Senate, the faculty house masters and students of the University.”</t>
+          <t>Clause explainer</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>The disputed mark sits between 'the faculty house masters' and 'and students of the University'. If it is an original comma, students are their own required approver and nobody can sign off on their behalf (strong veto, the reading the student movement wants). If it is ink damage or a later blemish, 'the faculty house masters and students' reads as one bound group, and consulting the house masters can be treated as consulting the students (weak veto, the reading the administration wants).</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Optional.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Clause explainer</t>
+          <t>Submission</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The disputed mark sits between 'the faculty house masters' and 'and students of the University'. If it is an original comma, students are their own required approver and nobody can sign off on their behalf (strong veto, the reading the student movement wants). If it is ink damage or a later blemish, 'the faculty house masters and students' reads as one bound group, and consulting the house masters can be treated as consulting the students (weak veto, the reading the administration wants).</t>
-        </is>
-      </c>
+          <t>Out of questions</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>You have used your forty questions. The president needs an answer now.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Shown when the question budget runs out; the player must then submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ending</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>You name Mira Shah and the theatre scenery loft. The president sends the archivist emeritus, Ruth Halpern, to the loft with you. Inside the 'Spring Gala 2023' tube is the Charter in its protective sleeve. Mira, when found, admits she removed it and edited the log because she believed the examination copy was not the original. Then the hidden payoff: Halpern lays the recovered Charter beside the examination copy. The copy is a near-perfect replica, commissioned at enormous expense by Adrian Vale, Celia Park and Martin Ellison so that the disputed mark would read as a blot and no student vote would ever be required. It was to be displayed in a glass case in the renovated center as though it were the original. The examination goes ahead at six with the real Charter on the table. The replica becomes a historical artifact after all, labelled honestly.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Also shown in the debrief to players who did not solve it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ending</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Right person, wrong place</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>You identify who removed the Charter but not where it is. The examination begins at six without the original, and the replica is examined as though it were genuine.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ending</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Wrong</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Your explanation does not fit the strongest evidence. The person you named had a motive, but the timeline, the access record and the hiding-place clues point elsewhere. The examination proceeds with the wrong document.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2230,6 +2560,84 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The mystery</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Who removed the Commons Charter from the university archive last night, why did they do it, and where is it now?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>The solution</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Mira Shah, a graduate archival researcher, removed the Charter using her own legitimate credential at 8:42 p.m., then edited the archive access log at 9:17 p.m. to hide the removal. She did it because she was convinced the document being prepared for tonight's public examination is not the original: the newspaper photograph of the 'examination copy' shows a disputed mark with edges and shadow that do not match the surrounding ink, and a crease visible in older photographs is missing. She hid the Charter, rolled in its protective sleeve, inside a poster tube labelled 'Spring Gala 2023' that Jonah Reed gave her, and the tube is now in the student theatre's scenery loft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Person question</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Who removed it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Place question</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Where is it now?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2520,7 +2928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2968,7 +3376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5984,7 +6392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6031,7 +6439,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Stance</t>
+          <t>Position on the CCC</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -6600,7 +7008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6862,486 +7270,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Major clue group</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Clue</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Given by</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>MC1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>The Charter was in its blue archival folder, seal intact, at the end of the student forum at 7:45 p.m., and was returned to the archive cabinet.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Leo Martinez (Q8); Evan Cho (Q5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>MC1</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Mira Shah's graduate credential opened the archive at 8:42 p.m. It was an ordinary entry; the door and cabinet show no damage.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Mira Shah (Q1); Priya Nwosu (Q7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>C03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>MC1</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>The archive access log was edited at 9:17 p.m., after the archive closed at 9:00. Editing the log requires an archive credential, not a maintenance or administrative one.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Priya Nwosu (Q1); Sofia Alvarez (Q5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>MC1</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>No credential other than Mira's opened the archive between the forum and closing time.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Leo Martinez (Q3); Priya Nwosu (Q6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>C05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>MC1</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Mira left the archive area at about 8:50 p.m. carrying something flat inside a protective sleeve.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Leo Martinez (Q7); Sofia Alvarez (Q1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>MC2</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Mira has argued for months, in seminars and in print, that the disputed mark is an original comma, the reading that gives students a strong veto.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Mira Shah (Q2); Nia Williams (Q2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>C07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>MC2</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>In the newspaper photograph of the 'examination copy', the disputed mark has sharper edges and a different paper shadow than the surrounding ink.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Mira Shah (Q6); Sofia Alvarez (Q2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>MC2</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>A small crease near the mark, visible in older photographs of the Charter, is absent from the newspaper photograph.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Priya Nwosu (Q3); Sofia Alvarez (Q8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MC2</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Late in the preparations the event materials stopped saying 'the original Charter' and started saying 'the Charter'; Celia Park kept pressing for 'a clean answer' for the Board.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Leo Martinez (Q5); Hana Petrov (Q3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>C10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>MC2</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Mira told other students she wanted to make sure 'the experts examine the real object', and feared the original would be quietly swapped or lost after the event.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Hana Petrov (Q2); Nia Williams (Q3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>C11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>MC3</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>At about 8:50 p.m. Mira asked whether the theatre had a dry, light-proof place to keep paper.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Jonah Reed (Q1); Evan Cho (Q4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>C12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>MC3</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Jonah gave Mira an empty poster tube labelled 'Spring Gala 2023'.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Jonah Reed (Q3); Nia Williams (Q4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>C13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>MC3</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>At about 8:55 p.m. a long cardboard tube with theatre paint on one end was carried from the Commons toward the theatre.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Leo Martinez (Q4); Evan Cho (Q1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>MC3</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>The 'Spring Gala 2023' tube is now in the theatre scenery loft, and it is heavier than an empty tube should be.</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Jonah Reed (Q6); Sofia Alvarez (Q4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>MC3</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>After Mira's visit Jonah moved several tubes in the scenery loft and did not update the inventory sheet.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Jonah Reed (Q8); Hana Petrov (Q4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>MC4</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Mira and Jonah were seen talking near the theatre at about 8:52 p.m. It looked like a practical conversation about storage, not a confrontation.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Evan Cho (Q7); Nia Williams (Q8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>C17</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>MC4</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Mira and Jonah disagree about the renovation's details but share one goal: the Charter must not be damaged or lost.</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Jonah Reed (Q2); Hana Petrov (Q7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>C18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>MC4</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>The Charter's protective sleeve is missing along with it. Whoever took it handled it like a conservator, not a thief.</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Mira Shah (Q4); Priya Nwosu (Q4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>C19</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>MC4</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Members of the administrative steering group do not hold archive credentials; they reach the archive through the archivist's office, and none of them used it that night.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Mira Shah (Q5); Hana Petrov (Q8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>C20</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>MC4</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Mira said she would 'keep it safe until someone can compare the two'. She intends to return the Charter once the examination copy has been checked against it.</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Evan Cho (Q3); Nia Williams (Q6)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>